<commit_message>
Updated Selenium framework and test suites
</commit_message>
<xml_diff>
--- a/sprint/src/test/resources/TestData.xlsx
+++ b/sprint/src/test/resources/TestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\eclipse-workspace\sprint\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\git\sprint_Local_Repo\sprint\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D2D6EA-DE9F-40CE-BA70-24983F0C4BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8216D93F-66C3-4247-B41C-C42A57BD9356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="103">
   <si>
     <t>TC_ID</t>
   </si>
@@ -330,6 +330,9 @@
   </si>
   <si>
     <t>https://www.saucedemo.com/inventory.html</t>
+  </si>
+  <si>
+    <t>Checkout: Your Information</t>
   </si>
 </sst>
 </file>
@@ -1150,7 +1153,9 @@
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="F7" t="s">
+        <v>102</v>
+      </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="4" t="s">

</xml_diff>